<commit_message>
Update May running group assignments
</commit_message>
<xml_diff>
--- a/public/assets/나빌러닝 조별기준.xlsx
+++ b/public/assets/나빌러닝 조별기준.xlsx
@@ -1,41 +1,42 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\running-club-site\public\assets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561BEBC1-2BCB-43CE-85B0-D37D9F2F51E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="2370" yWindow="3300" windowWidth="15375" windowHeight="7785" xr2:uid="{D8C9CABB-E8EB-4A41-AD3F-DDEB5E72321B}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>워크시트</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>Sheet1</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>DONG HYUN SEO</dc:creator>
+  <cp:lastModifiedBy>DONG HYUN SEO</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-04-12T02:24:26Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-04-18T01:08:52Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t>나빌러닝 조별 기준 (가을 대회 목표 마라톤 기록)</t>
@@ -169,187 +170,15 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>문재연</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>박운정</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>안효정</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>정주연</t>
-    </r>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>김나영</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>송경애</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>이은주</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>현혜인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>조민경</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>장신영</t>
-    </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <t>문재연, 박운정, 안효정, 정주연, 송경애, 이은주, 현혜인</t>
+  </si>
+  <si>
+    <t>김나영, 조민경, 장신영</t>
   </si>
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -507,7 +336,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -822,7 +651,43 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\running-club-site\public\assets\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561BEBC1-2BCB-43CE-85B0-D37D9F2F51E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="2370" yWindow="3300" windowWidth="15375" windowHeight="7785" xr2:uid="{D8C9CABB-E8EB-4A41-AD3F-DDEB5E72321B}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A9284E-2FDB-4FD1-8DFE-183B76E440C8}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Update July group assignments and notices
</commit_message>
<xml_diff>
--- a/public/assets/나빌러닝 조별기준.xlsx
+++ b/public/assets/나빌러닝 조별기준.xlsx
@@ -87,7 +87,7 @@
     <t>6:00~6:40/km</t>
   </si>
   <si>
-    <t>김종선, 민선홍, 박정미</t>
+    <t>김종선, 민선홍, 박정미, 안효정</t>
   </si>
   <si>
     <t>D</t>
@@ -99,7 +99,7 @@
     <t>6:30~7:00/km</t>
   </si>
   <si>
-    <t>김수미, 이혜경, 김성균</t>
+    <t>김수미, 이혜경, 김성균, 박운정, 현혜인</t>
   </si>
   <si>
     <t>E</t>
@@ -170,10 +170,10 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>문재연, 박운정, 안효정, 정주연, 송경애, 이은주, 현혜인</t>
-  </si>
-  <si>
-    <t>김나영, 조민경, 장신영</t>
+    <t>문재연, 정주연, 송경애, 이은주, 조민경</t>
+  </si>
+  <si>
+    <t>김나영, 장신영</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Remove Hyojeong Ahn from July promotion
</commit_message>
<xml_diff>
--- a/public/assets/나빌러닝 조별기준.xlsx
+++ b/public/assets/나빌러닝 조별기준.xlsx
@@ -87,7 +87,7 @@
     <t>6:00~6:40/km</t>
   </si>
   <si>
-    <t>김종선, 민선홍, 박정미, 안효정</t>
+    <t>김종선, 민선홍, 박정미</t>
   </si>
   <si>
     <t>D</t>
@@ -99,7 +99,7 @@
     <t>6:30~7:00/km</t>
   </si>
   <si>
-    <t>김수미, 이혜경, 김성균, 박운정, 현혜인</t>
+    <t>김수미, 이혜경, 김성균, 안효정, 박운정, 현혜인</t>
   </si>
   <si>
     <t>E</t>

</xml_diff>